<commit_message>
Working on response to reviewers and citations
</commit_message>
<xml_diff>
--- a/Documentation/Reports and Papers/Isometric_Force_Test/Tables/CoefficientTable.xlsx
+++ b/Documentation/Reports and Papers/Isometric_Force_Test/Tables/CoefficientTable.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Ben\Documents\GitHub\Bipedal_Robot\Documentation\Reports and Papers\Isometric_Force_Test\Tables\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Github\Bipedal_Robot\Documentation\Reports and Papers\Isometric_Force_Test\Tables\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3571FF59-9E23-464A-A0F5-6E28BA7ECD3F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2730" yWindow="2730" windowWidth="17280" windowHeight="8925" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Coefficient table" sheetId="4" r:id="rId1"/>
@@ -773,7 +773,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="65">
+  <cellXfs count="64">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
@@ -831,104 +831,103 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" quotePrefix="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" quotePrefix="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" quotePrefix="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" quotePrefix="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" quotePrefix="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" quotePrefix="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1211,43 +1210,43 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CFED512C-20B1-4472-8C7D-BFE8EE5F9AB6}">
   <dimension ref="A1:I25"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="22.5546875" customWidth="1"/>
-    <col min="2" max="2" width="19.88671875" customWidth="1"/>
-    <col min="3" max="3" width="11.33203125" customWidth="1"/>
-    <col min="4" max="4" width="7.6640625" customWidth="1"/>
-    <col min="6" max="6" width="10.44140625" customWidth="1"/>
-    <col min="7" max="7" width="12.109375" customWidth="1"/>
-    <col min="8" max="8" width="12.6640625" customWidth="1"/>
-    <col min="9" max="9" width="10.44140625" customWidth="1"/>
+    <col min="1" max="1" width="22.5703125" customWidth="1"/>
+    <col min="2" max="2" width="19.85546875" customWidth="1"/>
+    <col min="3" max="3" width="11.28515625" customWidth="1"/>
+    <col min="4" max="4" width="7.7109375" customWidth="1"/>
+    <col min="6" max="6" width="10.42578125" customWidth="1"/>
+    <col min="7" max="7" width="12.140625" customWidth="1"/>
+    <col min="8" max="8" width="12.7109375" customWidth="1"/>
+    <col min="9" max="9" width="10.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" s="3" customFormat="1" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="35" t="s">
+    <row r="1" spans="1:9" s="3" customFormat="1" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="46" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="35" t="s">
+      <c r="B1" s="46" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="35" t="s">
+      <c r="C1" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="D1" s="37" t="s">
+      <c r="D1" s="48" t="s">
         <v>9</v>
       </c>
-      <c r="E1" s="38"/>
-      <c r="F1" s="39"/>
-      <c r="G1" s="37" t="s">
+      <c r="E1" s="49"/>
+      <c r="F1" s="50"/>
+      <c r="G1" s="48" t="s">
         <v>3</v>
       </c>
-      <c r="H1" s="38"/>
-      <c r="I1" s="40"/>
-    </row>
-    <row r="2" spans="1:9" s="3" customFormat="1" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="36"/>
-      <c r="B2" s="36"/>
-      <c r="C2" s="36"/>
+      <c r="H1" s="49"/>
+      <c r="I1" s="51"/>
+    </row>
+    <row r="2" spans="1:9" s="3" customFormat="1" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="47"/>
+      <c r="B2" s="47"/>
+      <c r="C2" s="47"/>
       <c r="D2" s="4" t="s">
         <v>15</v>
       </c>
@@ -1267,8 +1266,8 @@
         <v>14</v>
       </c>
     </row>
-    <row r="3" spans="1:9" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="25" t="s">
+    <row r="3" spans="1:9" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="40" t="s">
         <v>6</v>
       </c>
       <c r="B3" s="1" t="s">
@@ -1277,42 +1276,42 @@
       <c r="C3" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="D3" s="27">
+      <c r="D3" s="36">
         <v>0.98319999999999996</v>
       </c>
-      <c r="E3" s="27">
+      <c r="E3" s="36">
         <v>13.62</v>
       </c>
-      <c r="F3" s="27" t="s">
+      <c r="F3" s="36" t="s">
         <v>44</v>
       </c>
-      <c r="G3" s="42" t="s">
+      <c r="G3" s="34" t="s">
         <v>4</v>
       </c>
-      <c r="H3" s="42" t="s">
+      <c r="H3" s="34" t="s">
         <v>4</v>
       </c>
-      <c r="I3" s="42" t="s">
+      <c r="I3" s="34" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="4" spans="1:9" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="26"/>
+    <row r="4" spans="1:9" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="42"/>
       <c r="B4" s="2" t="s">
         <v>55</v>
       </c>
       <c r="C4" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="D4" s="28"/>
-      <c r="E4" s="28"/>
-      <c r="F4" s="28"/>
-      <c r="G4" s="34"/>
-      <c r="H4" s="34"/>
-      <c r="I4" s="34"/>
-    </row>
-    <row r="5" spans="1:9" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="25" t="s">
+      <c r="D4" s="38"/>
+      <c r="E4" s="38"/>
+      <c r="F4" s="38"/>
+      <c r="G4" s="35"/>
+      <c r="H4" s="35"/>
+      <c r="I4" s="35"/>
+    </row>
+    <row r="5" spans="1:9" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="40" t="s">
         <v>7</v>
       </c>
       <c r="B5" s="1" t="s">
@@ -1321,42 +1320,42 @@
       <c r="C5" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="D5" s="25">
+      <c r="D5" s="40">
         <v>0.98680000000000001</v>
       </c>
-      <c r="E5" s="25" t="s">
+      <c r="E5" s="40" t="s">
         <v>47</v>
       </c>
-      <c r="F5" s="25" t="s">
+      <c r="F5" s="40" t="s">
         <v>44</v>
       </c>
-      <c r="G5" s="33">
+      <c r="G5" s="39">
         <v>0.92200000000000004</v>
       </c>
-      <c r="H5" s="33" t="s">
+      <c r="H5" s="39" t="s">
         <v>42</v>
       </c>
-      <c r="I5" s="33" t="s">
+      <c r="I5" s="39" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="6" spans="1:9" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="26"/>
+    <row r="6" spans="1:9" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="42"/>
       <c r="B6" s="2" t="s">
         <v>56</v>
       </c>
       <c r="C6" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="D6" s="26"/>
-      <c r="E6" s="26"/>
-      <c r="F6" s="26"/>
-      <c r="G6" s="34"/>
-      <c r="H6" s="34"/>
-      <c r="I6" s="34"/>
-    </row>
-    <row r="7" spans="1:9" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="33" t="s">
+      <c r="D6" s="42"/>
+      <c r="E6" s="42"/>
+      <c r="F6" s="42"/>
+      <c r="G6" s="35"/>
+      <c r="H6" s="35"/>
+      <c r="I6" s="35"/>
+    </row>
+    <row r="7" spans="1:9" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="39" t="s">
         <v>10</v>
       </c>
       <c r="B7" s="1" t="s">
@@ -1365,42 +1364,42 @@
       <c r="C7" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="D7" s="33">
+      <c r="D7" s="39">
         <v>0.99270000000000003</v>
       </c>
-      <c r="E7" s="33" t="s">
+      <c r="E7" s="39" t="s">
         <v>50</v>
       </c>
-      <c r="F7" s="33" t="s">
+      <c r="F7" s="39" t="s">
         <v>51</v>
       </c>
-      <c r="G7" s="42" t="s">
+      <c r="G7" s="34" t="s">
         <v>4</v>
       </c>
-      <c r="H7" s="42" t="s">
+      <c r="H7" s="34" t="s">
         <v>4</v>
       </c>
-      <c r="I7" s="42" t="s">
+      <c r="I7" s="34" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="8" spans="1:9" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="34"/>
+    <row r="8" spans="1:9" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="35"/>
       <c r="B8" s="2" t="s">
         <v>49</v>
       </c>
       <c r="C8" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="D8" s="34"/>
-      <c r="E8" s="34"/>
-      <c r="F8" s="34"/>
-      <c r="G8" s="34"/>
-      <c r="H8" s="34"/>
-      <c r="I8" s="34"/>
-    </row>
-    <row r="9" spans="1:9" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="29" t="s">
+      <c r="D8" s="35"/>
+      <c r="E8" s="35"/>
+      <c r="F8" s="35"/>
+      <c r="G8" s="35"/>
+      <c r="H8" s="35"/>
+      <c r="I8" s="35"/>
+    </row>
+    <row r="9" spans="1:9" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="43" t="s">
         <v>13</v>
       </c>
       <c r="B9" s="5" t="s">
@@ -1409,57 +1408,57 @@
       <c r="C9" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="D9" s="25">
+      <c r="D9" s="40">
         <v>0.99450000000000005</v>
       </c>
-      <c r="E9" s="25">
+      <c r="E9" s="40">
         <v>2.657E-2</v>
       </c>
-      <c r="F9" s="25" t="s">
+      <c r="F9" s="40" t="s">
         <v>33</v>
       </c>
-      <c r="G9" s="27">
+      <c r="G9" s="36">
         <v>0.98260000000000003</v>
       </c>
-      <c r="H9" s="27">
+      <c r="H9" s="36">
         <v>4.65E-2</v>
       </c>
-      <c r="I9" s="27" t="s">
+      <c r="I9" s="36" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="10" spans="1:9" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="30"/>
+    <row r="10" spans="1:9" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="44"/>
       <c r="B10" s="5" t="s">
         <v>27</v>
       </c>
       <c r="C10" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="D10" s="32"/>
-      <c r="E10" s="32"/>
-      <c r="F10" s="32"/>
-      <c r="G10" s="41"/>
-      <c r="H10" s="41"/>
-      <c r="I10" s="41"/>
-    </row>
-    <row r="11" spans="1:9" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="31"/>
+      <c r="D10" s="41"/>
+      <c r="E10" s="41"/>
+      <c r="F10" s="41"/>
+      <c r="G10" s="37"/>
+      <c r="H10" s="37"/>
+      <c r="I10" s="37"/>
+    </row>
+    <row r="11" spans="1:9" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="45"/>
       <c r="B11" s="5" t="s">
         <v>28</v>
       </c>
       <c r="C11" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="D11" s="26"/>
-      <c r="E11" s="26"/>
-      <c r="F11" s="26"/>
-      <c r="G11" s="28"/>
-      <c r="H11" s="28"/>
-      <c r="I11" s="28"/>
-    </row>
-    <row r="12" spans="1:9" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="29" t="s">
+      <c r="D11" s="42"/>
+      <c r="E11" s="42"/>
+      <c r="F11" s="42"/>
+      <c r="G11" s="38"/>
+      <c r="H11" s="38"/>
+      <c r="I11" s="38"/>
+    </row>
+    <row r="12" spans="1:9" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="43" t="s">
         <v>11</v>
       </c>
       <c r="B12" s="5" t="s">
@@ -1468,57 +1467,57 @@
       <c r="C12" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="D12" s="25">
+      <c r="D12" s="40">
         <v>0.99580000000000002</v>
       </c>
-      <c r="E12" s="25">
+      <c r="E12" s="40">
         <v>2.2679999999999999E-2</v>
       </c>
-      <c r="F12" s="25" t="s">
+      <c r="F12" s="40" t="s">
         <v>24</v>
       </c>
-      <c r="G12" s="27">
+      <c r="G12" s="36">
         <v>0.98839999999999995</v>
       </c>
-      <c r="H12" s="27">
+      <c r="H12" s="36">
         <v>3.8739999999999997E-2</v>
       </c>
-      <c r="I12" s="27" t="s">
+      <c r="I12" s="36" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="13" spans="1:9" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="30"/>
+    <row r="13" spans="1:9" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="44"/>
       <c r="B13" s="5" t="s">
         <v>35</v>
       </c>
       <c r="C13" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="D13" s="32"/>
-      <c r="E13" s="32"/>
-      <c r="F13" s="32"/>
-      <c r="G13" s="41"/>
-      <c r="H13" s="41"/>
-      <c r="I13" s="41"/>
-    </row>
-    <row r="14" spans="1:9" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="31"/>
+      <c r="D13" s="41"/>
+      <c r="E13" s="41"/>
+      <c r="F13" s="41"/>
+      <c r="G13" s="37"/>
+      <c r="H13" s="37"/>
+      <c r="I13" s="37"/>
+    </row>
+    <row r="14" spans="1:9" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="45"/>
       <c r="B14" s="5" t="s">
         <v>34</v>
       </c>
       <c r="C14" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="D14" s="26"/>
-      <c r="E14" s="26"/>
-      <c r="F14" s="26"/>
-      <c r="G14" s="28"/>
-      <c r="H14" s="28"/>
-      <c r="I14" s="28"/>
-    </row>
-    <row r="15" spans="1:9" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="25" t="s">
+      <c r="D14" s="42"/>
+      <c r="E14" s="42"/>
+      <c r="F14" s="42"/>
+      <c r="G14" s="38"/>
+      <c r="H14" s="38"/>
+      <c r="I14" s="38"/>
+    </row>
+    <row r="15" spans="1:9" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="40" t="s">
         <v>5</v>
       </c>
       <c r="B15" s="5" t="s">
@@ -1527,57 +1526,57 @@
       <c r="C15" s="5" t="s">
         <v>60</v>
       </c>
-      <c r="D15" s="25">
+      <c r="D15" s="40">
         <v>0.99590000000000001</v>
       </c>
-      <c r="E15" s="25">
+      <c r="E15" s="40">
         <v>1.8380000000000001E-2</v>
       </c>
-      <c r="F15" s="25" t="s">
+      <c r="F15" s="40" t="s">
         <v>20</v>
       </c>
-      <c r="G15" s="27" t="s">
+      <c r="G15" s="36" t="s">
         <v>4</v>
       </c>
-      <c r="H15" s="27" t="s">
+      <c r="H15" s="36" t="s">
         <v>4</v>
       </c>
-      <c r="I15" s="27" t="s">
+      <c r="I15" s="36" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="16" spans="1:9" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="32"/>
+    <row r="16" spans="1:9" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="41"/>
       <c r="B16" s="5" t="s">
         <v>58</v>
       </c>
       <c r="C16" s="5" t="s">
         <v>61</v>
       </c>
-      <c r="D16" s="32"/>
-      <c r="E16" s="32"/>
-      <c r="F16" s="32"/>
-      <c r="G16" s="41"/>
-      <c r="H16" s="41"/>
-      <c r="I16" s="41"/>
-    </row>
-    <row r="17" spans="1:9" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="26"/>
+      <c r="D16" s="41"/>
+      <c r="E16" s="41"/>
+      <c r="F16" s="41"/>
+      <c r="G16" s="37"/>
+      <c r="H16" s="37"/>
+      <c r="I16" s="37"/>
+    </row>
+    <row r="17" spans="1:9" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="42"/>
       <c r="B17" s="5" t="s">
         <v>59</v>
       </c>
       <c r="C17" s="5" t="s">
         <v>62</v>
       </c>
-      <c r="D17" s="26"/>
-      <c r="E17" s="26"/>
-      <c r="F17" s="26"/>
-      <c r="G17" s="28"/>
-      <c r="H17" s="28"/>
-      <c r="I17" s="28"/>
-    </row>
-    <row r="18" spans="1:9" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="25" t="s">
+      <c r="D17" s="42"/>
+      <c r="E17" s="42"/>
+      <c r="F17" s="42"/>
+      <c r="G17" s="38"/>
+      <c r="H17" s="38"/>
+      <c r="I17" s="38"/>
+    </row>
+    <row r="18" spans="1:9" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="40" t="s">
         <v>8</v>
       </c>
       <c r="B18" s="5" t="s">
@@ -1586,56 +1585,56 @@
       <c r="C18" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="D18" s="25">
+      <c r="D18" s="40">
         <v>0.98529999999999995</v>
       </c>
-      <c r="E18" s="25">
+      <c r="E18" s="40">
         <v>3.7539999999999997E-2</v>
       </c>
-      <c r="F18" s="25" t="s">
+      <c r="F18" s="40" t="s">
         <v>19</v>
       </c>
-      <c r="G18" s="27" t="s">
+      <c r="G18" s="36" t="s">
         <v>4</v>
       </c>
-      <c r="H18" s="27" t="s">
+      <c r="H18" s="36" t="s">
         <v>4</v>
       </c>
-      <c r="I18" s="27" t="s">
+      <c r="I18" s="36" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="19" spans="1:9" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="32"/>
+    <row r="19" spans="1:9" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="41"/>
       <c r="B19" s="5" t="s">
         <v>17</v>
       </c>
       <c r="C19" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="D19" s="32"/>
-      <c r="E19" s="32"/>
-      <c r="F19" s="32"/>
-      <c r="G19" s="41"/>
-      <c r="H19" s="41"/>
-      <c r="I19" s="41"/>
-    </row>
-    <row r="20" spans="1:9" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="26"/>
+      <c r="D19" s="41"/>
+      <c r="E19" s="41"/>
+      <c r="F19" s="41"/>
+      <c r="G19" s="37"/>
+      <c r="H19" s="37"/>
+      <c r="I19" s="37"/>
+    </row>
+    <row r="20" spans="1:9" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="42"/>
       <c r="B20" s="5" t="s">
         <v>18</v>
       </c>
       <c r="C20" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="D20" s="26"/>
-      <c r="E20" s="26"/>
-      <c r="F20" s="26"/>
-      <c r="G20" s="28"/>
-      <c r="H20" s="28"/>
-      <c r="I20" s="28"/>
-    </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="D20" s="42"/>
+      <c r="E20" s="42"/>
+      <c r="F20" s="42"/>
+      <c r="G20" s="38"/>
+      <c r="H20" s="38"/>
+      <c r="I20" s="38"/>
+    </row>
+    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A21" s="7"/>
       <c r="B21" s="7"/>
       <c r="C21" s="7"/>
@@ -1643,7 +1642,7 @@
       <c r="E21" s="8"/>
       <c r="F21" s="8"/>
     </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A22" s="7"/>
       <c r="B22" s="7"/>
       <c r="C22" s="7"/>
@@ -1651,7 +1650,7 @@
       <c r="E22" s="8"/>
       <c r="F22" s="8"/>
     </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A23" s="7"/>
       <c r="B23" s="7"/>
       <c r="C23" s="7"/>
@@ -1659,7 +1658,7 @@
       <c r="E23" s="8"/>
       <c r="F23" s="8"/>
     </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A24" s="7"/>
       <c r="B24" s="7"/>
       <c r="C24" s="7"/>
@@ -1667,7 +1666,7 @@
       <c r="E24" s="8"/>
       <c r="F24" s="8"/>
     </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A25" s="7"/>
       <c r="B25" s="7"/>
       <c r="C25" s="7"/>
@@ -1677,6 +1676,44 @@
     </row>
   </sheetData>
   <mergeCells count="54">
+    <mergeCell ref="A3:A4"/>
+    <mergeCell ref="D3:D4"/>
+    <mergeCell ref="E3:E4"/>
+    <mergeCell ref="F3:F4"/>
+    <mergeCell ref="A5:A6"/>
+    <mergeCell ref="D5:D6"/>
+    <mergeCell ref="E5:E6"/>
+    <mergeCell ref="A9:A11"/>
+    <mergeCell ref="D9:D11"/>
+    <mergeCell ref="E9:E11"/>
+    <mergeCell ref="F9:F11"/>
+    <mergeCell ref="F5:F6"/>
+    <mergeCell ref="D7:D8"/>
+    <mergeCell ref="E7:E8"/>
+    <mergeCell ref="F7:F8"/>
+    <mergeCell ref="A7:A8"/>
+    <mergeCell ref="B1:B2"/>
+    <mergeCell ref="C1:C2"/>
+    <mergeCell ref="D1:F1"/>
+    <mergeCell ref="G1:I1"/>
+    <mergeCell ref="A1:A2"/>
+    <mergeCell ref="A12:A14"/>
+    <mergeCell ref="D12:D14"/>
+    <mergeCell ref="E12:E14"/>
+    <mergeCell ref="F12:F14"/>
+    <mergeCell ref="G12:G14"/>
+    <mergeCell ref="H18:H20"/>
+    <mergeCell ref="I18:I20"/>
+    <mergeCell ref="A15:A17"/>
+    <mergeCell ref="D15:D17"/>
+    <mergeCell ref="E15:E17"/>
+    <mergeCell ref="F15:F17"/>
+    <mergeCell ref="G15:G17"/>
+    <mergeCell ref="A18:A20"/>
+    <mergeCell ref="D18:D20"/>
+    <mergeCell ref="E18:E20"/>
+    <mergeCell ref="F18:F20"/>
+    <mergeCell ref="G18:G20"/>
     <mergeCell ref="G3:G4"/>
     <mergeCell ref="H3:H4"/>
     <mergeCell ref="I3:I4"/>
@@ -1693,44 +1730,6 @@
     <mergeCell ref="G7:G8"/>
     <mergeCell ref="H7:H8"/>
     <mergeCell ref="I7:I8"/>
-    <mergeCell ref="H18:H20"/>
-    <mergeCell ref="I18:I20"/>
-    <mergeCell ref="A15:A17"/>
-    <mergeCell ref="D15:D17"/>
-    <mergeCell ref="E15:E17"/>
-    <mergeCell ref="F15:F17"/>
-    <mergeCell ref="G15:G17"/>
-    <mergeCell ref="A18:A20"/>
-    <mergeCell ref="D18:D20"/>
-    <mergeCell ref="E18:E20"/>
-    <mergeCell ref="F18:F20"/>
-    <mergeCell ref="G18:G20"/>
-    <mergeCell ref="A12:A14"/>
-    <mergeCell ref="D12:D14"/>
-    <mergeCell ref="E12:E14"/>
-    <mergeCell ref="F12:F14"/>
-    <mergeCell ref="G12:G14"/>
-    <mergeCell ref="B1:B2"/>
-    <mergeCell ref="C1:C2"/>
-    <mergeCell ref="D1:F1"/>
-    <mergeCell ref="G1:I1"/>
-    <mergeCell ref="A1:A2"/>
-    <mergeCell ref="A9:A11"/>
-    <mergeCell ref="D9:D11"/>
-    <mergeCell ref="E9:E11"/>
-    <mergeCell ref="F9:F11"/>
-    <mergeCell ref="F5:F6"/>
-    <mergeCell ref="D7:D8"/>
-    <mergeCell ref="E7:E8"/>
-    <mergeCell ref="F7:F8"/>
-    <mergeCell ref="A7:A8"/>
-    <mergeCell ref="A3:A4"/>
-    <mergeCell ref="D3:D4"/>
-    <mergeCell ref="E3:E4"/>
-    <mergeCell ref="F3:F4"/>
-    <mergeCell ref="A5:A6"/>
-    <mergeCell ref="D5:D6"/>
-    <mergeCell ref="E5:E6"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
@@ -1740,43 +1739,43 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{248EE269-D9C6-4699-8B6A-E13E54F18600}">
   <dimension ref="A1:J17"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="22.5546875" customWidth="1"/>
+    <col min="1" max="1" width="22.5703125" customWidth="1"/>
     <col min="2" max="2" width="18" customWidth="1"/>
     <col min="3" max="3" width="17" customWidth="1"/>
-    <col min="4" max="4" width="14.33203125" customWidth="1"/>
-    <col min="5" max="5" width="9.33203125" customWidth="1"/>
-    <col min="6" max="6" width="10.44140625" customWidth="1"/>
-    <col min="8" max="8" width="12.109375" customWidth="1"/>
-    <col min="9" max="9" width="11.44140625" customWidth="1"/>
+    <col min="4" max="4" width="14.28515625" customWidth="1"/>
+    <col min="5" max="5" width="9.28515625" customWidth="1"/>
+    <col min="6" max="6" width="10.42578125" customWidth="1"/>
+    <col min="8" max="8" width="12.140625" customWidth="1"/>
+    <col min="9" max="9" width="11.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" s="3" customFormat="1" ht="28.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="35" t="s">
+    <row r="1" spans="1:10" s="3" customFormat="1" ht="28.15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="46" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="35" t="s">
+      <c r="B1" s="46" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="35" t="s">
+      <c r="C1" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="D1" s="43" t="s">
+      <c r="D1" s="52" t="s">
         <v>9</v>
       </c>
-      <c r="E1" s="44"/>
-      <c r="F1" s="46"/>
-      <c r="G1" s="43" t="s">
+      <c r="E1" s="53"/>
+      <c r="F1" s="55"/>
+      <c r="G1" s="52" t="s">
         <v>3</v>
       </c>
-      <c r="H1" s="44"/>
-      <c r="I1" s="45"/>
-    </row>
-    <row r="2" spans="1:10" s="3" customFormat="1" ht="28.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="36"/>
-      <c r="B2" s="36"/>
-      <c r="C2" s="36"/>
+      <c r="H1" s="53"/>
+      <c r="I1" s="54"/>
+    </row>
+    <row r="2" spans="1:10" s="3" customFormat="1" ht="28.15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="47"/>
+      <c r="B2" s="47"/>
+      <c r="C2" s="47"/>
       <c r="D2" s="6" t="s">
         <v>102</v>
       </c>
@@ -1796,8 +1795,8 @@
         <v>14</v>
       </c>
     </row>
-    <row r="3" spans="1:10" ht="28.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="29" t="s">
+    <row r="3" spans="1:10" ht="28.15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="43" t="s">
         <v>134</v>
       </c>
       <c r="B3" s="5" t="s">
@@ -1806,60 +1805,60 @@
       <c r="C3" s="5" t="s">
         <v>118</v>
       </c>
-      <c r="D3" s="25">
+      <c r="D3" s="40">
         <v>0.99480000000000002</v>
       </c>
-      <c r="E3" s="25">
+      <c r="E3" s="40">
         <v>2.5829999999999999E-2</v>
       </c>
-      <c r="F3" s="25" t="s">
+      <c r="F3" s="40" t="s">
         <v>33</v>
       </c>
-      <c r="G3" s="27">
+      <c r="G3" s="36">
         <v>0.98819999999999997</v>
       </c>
-      <c r="H3" s="27">
+      <c r="H3" s="36">
         <v>3.8769999999999999E-2</v>
       </c>
-      <c r="I3" s="27" t="s">
+      <c r="I3" s="36" t="s">
         <v>77</v>
       </c>
       <c r="J3" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="4" spans="1:10" ht="28.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="30"/>
+    <row r="4" spans="1:10" ht="28.15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="44"/>
       <c r="B4" s="5" t="s">
         <v>120</v>
       </c>
       <c r="C4" s="5" t="s">
         <v>79</v>
       </c>
-      <c r="D4" s="32"/>
-      <c r="E4" s="32"/>
-      <c r="F4" s="32"/>
-      <c r="G4" s="41"/>
-      <c r="H4" s="41"/>
-      <c r="I4" s="41"/>
-    </row>
-    <row r="5" spans="1:10" ht="28.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="31"/>
+      <c r="D4" s="41"/>
+      <c r="E4" s="41"/>
+      <c r="F4" s="41"/>
+      <c r="G4" s="37"/>
+      <c r="H4" s="37"/>
+      <c r="I4" s="37"/>
+    </row>
+    <row r="5" spans="1:10" ht="28.15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="45"/>
       <c r="B5" s="5" t="s">
         <v>121</v>
       </c>
       <c r="C5" s="5" t="s">
         <v>78</v>
       </c>
-      <c r="D5" s="26"/>
-      <c r="E5" s="26"/>
-      <c r="F5" s="26"/>
-      <c r="G5" s="28"/>
-      <c r="H5" s="28"/>
-      <c r="I5" s="28"/>
-    </row>
-    <row r="6" spans="1:10" ht="28.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="29" t="s">
+      <c r="D5" s="42"/>
+      <c r="E5" s="42"/>
+      <c r="F5" s="42"/>
+      <c r="G5" s="38"/>
+      <c r="H5" s="38"/>
+      <c r="I5" s="38"/>
+    </row>
+    <row r="6" spans="1:10" ht="28.15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="43" t="s">
         <v>135</v>
       </c>
       <c r="B6" s="5" t="s">
@@ -1868,60 +1867,60 @@
       <c r="C6" s="5" t="s">
         <v>117</v>
       </c>
-      <c r="D6" s="25">
+      <c r="D6" s="40">
         <v>0.99980000000000002</v>
       </c>
-      <c r="E6" s="25">
+      <c r="E6" s="40">
         <v>4.5370000000000002E-3</v>
       </c>
-      <c r="F6" s="25" t="s">
+      <c r="F6" s="40" t="s">
         <v>80</v>
       </c>
-      <c r="G6" s="27">
+      <c r="G6" s="36">
         <v>0.98780000000000001</v>
       </c>
-      <c r="H6" s="27">
+      <c r="H6" s="36">
         <v>3.9660000000000001E-2</v>
       </c>
-      <c r="I6" s="27" t="s">
+      <c r="I6" s="36" t="s">
         <v>81</v>
       </c>
       <c r="J6" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="7" spans="1:10" ht="28.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="30"/>
+    <row r="7" spans="1:10" ht="28.15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="44"/>
       <c r="B7" s="5" t="s">
         <v>123</v>
       </c>
       <c r="C7" s="5" t="s">
         <v>82</v>
       </c>
-      <c r="D7" s="32"/>
-      <c r="E7" s="32"/>
-      <c r="F7" s="32"/>
-      <c r="G7" s="41"/>
-      <c r="H7" s="41"/>
-      <c r="I7" s="41"/>
-    </row>
-    <row r="8" spans="1:10" ht="28.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="31"/>
+      <c r="D7" s="41"/>
+      <c r="E7" s="41"/>
+      <c r="F7" s="41"/>
+      <c r="G7" s="37"/>
+      <c r="H7" s="37"/>
+      <c r="I7" s="37"/>
+    </row>
+    <row r="8" spans="1:10" ht="28.15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="45"/>
       <c r="B8" s="5" t="s">
         <v>124</v>
       </c>
       <c r="C8" s="5" t="s">
         <v>83</v>
       </c>
-      <c r="D8" s="26"/>
-      <c r="E8" s="26"/>
-      <c r="F8" s="26"/>
-      <c r="G8" s="28"/>
-      <c r="H8" s="28"/>
-      <c r="I8" s="28"/>
-    </row>
-    <row r="9" spans="1:10" ht="28.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="25" t="s">
+      <c r="D8" s="42"/>
+      <c r="E8" s="42"/>
+      <c r="F8" s="42"/>
+      <c r="G8" s="38"/>
+      <c r="H8" s="38"/>
+      <c r="I8" s="38"/>
+    </row>
+    <row r="9" spans="1:10" ht="28.15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="40" t="s">
         <v>136</v>
       </c>
       <c r="B9" s="5" t="s">
@@ -1930,60 +1929,60 @@
       <c r="C9" s="5" t="s">
         <v>109</v>
       </c>
-      <c r="D9" s="25">
+      <c r="D9" s="40">
         <v>0.99519999999999997</v>
       </c>
-      <c r="E9" s="25">
+      <c r="E9" s="40">
         <v>1.992E-2</v>
       </c>
-      <c r="F9" s="25" t="s">
+      <c r="F9" s="40" t="s">
         <v>104</v>
       </c>
-      <c r="G9" s="27">
+      <c r="G9" s="36">
         <v>0.99039999999999995</v>
       </c>
-      <c r="H9" s="27">
+      <c r="H9" s="36">
         <v>2.6259999999999999E-2</v>
       </c>
-      <c r="I9" s="27" t="s">
+      <c r="I9" s="36" t="s">
         <v>105</v>
       </c>
       <c r="J9" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="10" spans="1:10" ht="28.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="32"/>
+    <row r="10" spans="1:10" ht="28.15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="41"/>
       <c r="B10" s="5" t="s">
         <v>126</v>
       </c>
       <c r="C10" s="5" t="s">
         <v>110</v>
       </c>
-      <c r="D10" s="32"/>
-      <c r="E10" s="32"/>
-      <c r="F10" s="32"/>
-      <c r="G10" s="41"/>
-      <c r="H10" s="41"/>
-      <c r="I10" s="41"/>
-    </row>
-    <row r="11" spans="1:10" ht="28.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="26"/>
+      <c r="D10" s="41"/>
+      <c r="E10" s="41"/>
+      <c r="F10" s="41"/>
+      <c r="G10" s="37"/>
+      <c r="H10" s="37"/>
+      <c r="I10" s="37"/>
+    </row>
+    <row r="11" spans="1:10" ht="28.15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="42"/>
       <c r="B11" s="5" t="s">
         <v>127</v>
       </c>
       <c r="C11" s="5" t="s">
         <v>111</v>
       </c>
-      <c r="D11" s="26"/>
-      <c r="E11" s="26"/>
-      <c r="F11" s="26"/>
-      <c r="G11" s="28"/>
-      <c r="H11" s="28"/>
-      <c r="I11" s="28"/>
-    </row>
-    <row r="12" spans="1:10" ht="28.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="25" t="s">
+      <c r="D11" s="42"/>
+      <c r="E11" s="42"/>
+      <c r="F11" s="42"/>
+      <c r="G11" s="38"/>
+      <c r="H11" s="38"/>
+      <c r="I11" s="38"/>
+    </row>
+    <row r="12" spans="1:10" ht="28.15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="40" t="s">
         <v>137</v>
       </c>
       <c r="B12" s="5" t="s">
@@ -1992,60 +1991,60 @@
       <c r="C12" s="5" t="s">
         <v>106</v>
       </c>
-      <c r="D12" s="25">
+      <c r="D12" s="40">
         <v>0.99270000000000003</v>
       </c>
-      <c r="E12" s="25">
+      <c r="E12" s="40">
         <v>2.291E-2</v>
       </c>
-      <c r="F12" s="25" t="s">
+      <c r="F12" s="40" t="s">
         <v>33</v>
       </c>
-      <c r="G12" s="27">
+      <c r="G12" s="36">
         <v>0.995</v>
       </c>
-      <c r="H12" s="27">
+      <c r="H12" s="36">
         <v>2.019E-2</v>
       </c>
-      <c r="I12" s="27" t="s">
+      <c r="I12" s="36" t="s">
         <v>65</v>
       </c>
       <c r="J12" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="13" spans="1:10" ht="28.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="32"/>
+    <row r="13" spans="1:10" ht="28.15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="41"/>
       <c r="B13" s="5" t="s">
         <v>129</v>
       </c>
       <c r="C13" s="5" t="s">
         <v>107</v>
       </c>
-      <c r="D13" s="32"/>
-      <c r="E13" s="32"/>
-      <c r="F13" s="32"/>
-      <c r="G13" s="41"/>
-      <c r="H13" s="41"/>
-      <c r="I13" s="41"/>
-    </row>
-    <row r="14" spans="1:10" ht="28.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="26"/>
+      <c r="D13" s="41"/>
+      <c r="E13" s="41"/>
+      <c r="F13" s="41"/>
+      <c r="G13" s="37"/>
+      <c r="H13" s="37"/>
+      <c r="I13" s="37"/>
+    </row>
+    <row r="14" spans="1:10" ht="28.15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="42"/>
       <c r="B14" s="5" t="s">
         <v>130</v>
       </c>
       <c r="C14" s="5" t="s">
         <v>108</v>
       </c>
-      <c r="D14" s="26"/>
-      <c r="E14" s="26"/>
-      <c r="F14" s="26"/>
-      <c r="G14" s="28"/>
-      <c r="H14" s="28"/>
-      <c r="I14" s="28"/>
-    </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A15" s="25" t="s">
+      <c r="D14" s="42"/>
+      <c r="E14" s="42"/>
+      <c r="F14" s="42"/>
+      <c r="G14" s="38"/>
+      <c r="H14" s="38"/>
+      <c r="I14" s="38"/>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A15" s="40" t="s">
         <v>116</v>
       </c>
       <c r="B15" s="5" t="s">
@@ -2054,65 +2053,87 @@
       <c r="C15" s="5" t="s">
         <v>112</v>
       </c>
-      <c r="D15" s="25">
+      <c r="D15" s="40">
         <v>0.98340000000000005</v>
       </c>
-      <c r="E15" s="25">
+      <c r="E15" s="40">
         <v>3.9109999999999999E-2</v>
       </c>
-      <c r="F15" s="25" t="s">
+      <c r="F15" s="40" t="s">
         <v>115</v>
       </c>
-      <c r="G15" s="27" t="s">
+      <c r="G15" s="36" t="s">
         <v>4</v>
       </c>
-      <c r="H15" s="27" t="s">
+      <c r="H15" s="36" t="s">
         <v>4</v>
       </c>
-      <c r="I15" s="27" t="s">
+      <c r="I15" s="36" t="s">
         <v>4</v>
       </c>
       <c r="J15" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A16" s="32"/>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A16" s="41"/>
       <c r="B16" s="5" t="s">
         <v>132</v>
       </c>
       <c r="C16" s="5" t="s">
         <v>113</v>
       </c>
-      <c r="D16" s="32"/>
-      <c r="E16" s="32"/>
-      <c r="F16" s="32"/>
-      <c r="G16" s="41"/>
-      <c r="H16" s="41"/>
-      <c r="I16" s="41"/>
-    </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A17" s="26"/>
+      <c r="D16" s="41"/>
+      <c r="E16" s="41"/>
+      <c r="F16" s="41"/>
+      <c r="G16" s="37"/>
+      <c r="H16" s="37"/>
+      <c r="I16" s="37"/>
+    </row>
+    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A17" s="42"/>
       <c r="B17" s="5" t="s">
         <v>133</v>
       </c>
       <c r="C17" s="5" t="s">
         <v>114</v>
       </c>
-      <c r="D17" s="26"/>
-      <c r="E17" s="26"/>
-      <c r="F17" s="26"/>
-      <c r="G17" s="28"/>
-      <c r="H17" s="28"/>
-      <c r="I17" s="28"/>
+      <c r="D17" s="42"/>
+      <c r="E17" s="42"/>
+      <c r="F17" s="42"/>
+      <c r="G17" s="38"/>
+      <c r="H17" s="38"/>
+      <c r="I17" s="38"/>
     </row>
   </sheetData>
   <mergeCells count="40">
-    <mergeCell ref="I6:I8"/>
-    <mergeCell ref="I3:I5"/>
-    <mergeCell ref="H3:H5"/>
-    <mergeCell ref="G3:G5"/>
-    <mergeCell ref="F3:F5"/>
+    <mergeCell ref="H15:H17"/>
+    <mergeCell ref="I15:I17"/>
+    <mergeCell ref="A15:A17"/>
+    <mergeCell ref="D15:D17"/>
+    <mergeCell ref="E15:E17"/>
+    <mergeCell ref="F15:F17"/>
+    <mergeCell ref="G15:G17"/>
+    <mergeCell ref="A1:A2"/>
+    <mergeCell ref="G1:I1"/>
+    <mergeCell ref="B1:B2"/>
+    <mergeCell ref="C1:C2"/>
+    <mergeCell ref="D1:F1"/>
+    <mergeCell ref="E6:E8"/>
+    <mergeCell ref="F6:F8"/>
+    <mergeCell ref="G6:G8"/>
+    <mergeCell ref="H6:H8"/>
+    <mergeCell ref="E3:E5"/>
+    <mergeCell ref="I9:I11"/>
+    <mergeCell ref="H9:H11"/>
+    <mergeCell ref="G9:G11"/>
+    <mergeCell ref="F9:F11"/>
+    <mergeCell ref="E9:E11"/>
+    <mergeCell ref="E12:E14"/>
+    <mergeCell ref="F12:F14"/>
+    <mergeCell ref="G12:G14"/>
+    <mergeCell ref="H12:H14"/>
+    <mergeCell ref="I12:I14"/>
     <mergeCell ref="A3:A5"/>
     <mergeCell ref="D3:D5"/>
     <mergeCell ref="D6:D8"/>
@@ -2121,33 +2142,11 @@
     <mergeCell ref="A12:A14"/>
     <mergeCell ref="A9:A11"/>
     <mergeCell ref="A6:A8"/>
-    <mergeCell ref="E12:E14"/>
-    <mergeCell ref="F12:F14"/>
-    <mergeCell ref="G12:G14"/>
-    <mergeCell ref="H12:H14"/>
-    <mergeCell ref="I12:I14"/>
-    <mergeCell ref="I9:I11"/>
-    <mergeCell ref="H9:H11"/>
-    <mergeCell ref="G9:G11"/>
-    <mergeCell ref="F9:F11"/>
-    <mergeCell ref="E9:E11"/>
-    <mergeCell ref="E6:E8"/>
-    <mergeCell ref="F6:F8"/>
-    <mergeCell ref="G6:G8"/>
-    <mergeCell ref="H6:H8"/>
-    <mergeCell ref="E3:E5"/>
-    <mergeCell ref="A1:A2"/>
-    <mergeCell ref="G1:I1"/>
-    <mergeCell ref="B1:B2"/>
-    <mergeCell ref="C1:C2"/>
-    <mergeCell ref="D1:F1"/>
-    <mergeCell ref="H15:H17"/>
-    <mergeCell ref="I15:I17"/>
-    <mergeCell ref="A15:A17"/>
-    <mergeCell ref="D15:D17"/>
-    <mergeCell ref="E15:E17"/>
-    <mergeCell ref="F15:F17"/>
-    <mergeCell ref="G15:G17"/>
+    <mergeCell ref="I6:I8"/>
+    <mergeCell ref="I3:I5"/>
+    <mergeCell ref="H3:H5"/>
+    <mergeCell ref="G3:G5"/>
+    <mergeCell ref="F3:F5"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -2157,40 +2156,40 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{63494E59-DB24-4854-848F-7E392F2629DB}">
   <dimension ref="A1:J12"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="19.33203125" customWidth="1"/>
-    <col min="2" max="2" width="31.44140625" customWidth="1"/>
-    <col min="3" max="3" width="20.5546875" customWidth="1"/>
-    <col min="6" max="6" width="11.5546875" customWidth="1"/>
-    <col min="9" max="9" width="10.6640625" customWidth="1"/>
+    <col min="1" max="1" width="19.28515625" customWidth="1"/>
+    <col min="2" max="2" width="31.42578125" customWidth="1"/>
+    <col min="3" max="3" width="20.5703125" customWidth="1"/>
+    <col min="6" max="6" width="11.5703125" customWidth="1"/>
+    <col min="9" max="9" width="10.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="28.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="35" t="s">
+    <row r="1" spans="1:10" ht="28.15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="46" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="35" t="s">
+      <c r="B1" s="46" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="35" t="s">
+      <c r="C1" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="D1" s="43" t="s">
+      <c r="D1" s="52" t="s">
         <v>9</v>
       </c>
-      <c r="E1" s="44"/>
-      <c r="F1" s="46"/>
-      <c r="G1" s="43" t="s">
+      <c r="E1" s="53"/>
+      <c r="F1" s="55"/>
+      <c r="G1" s="52" t="s">
         <v>87</v>
       </c>
-      <c r="H1" s="44"/>
-      <c r="I1" s="45"/>
-    </row>
-    <row r="2" spans="1:10" ht="28.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="36"/>
-      <c r="B2" s="36"/>
-      <c r="C2" s="36"/>
+      <c r="H1" s="53"/>
+      <c r="I1" s="54"/>
+    </row>
+    <row r="2" spans="1:10" ht="28.15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="47"/>
+      <c r="B2" s="47"/>
+      <c r="C2" s="47"/>
       <c r="D2" s="6" t="s">
         <v>102</v>
       </c>
@@ -2210,8 +2209,8 @@
         <v>14</v>
       </c>
     </row>
-    <row r="3" spans="1:10" ht="28.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="47" t="s">
+    <row r="3" spans="1:10" ht="28.15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="56" t="s">
         <v>7</v>
       </c>
       <c r="B3" s="13" t="s">
@@ -2220,45 +2219,45 @@
       <c r="C3" s="14" t="s">
         <v>71</v>
       </c>
-      <c r="D3" s="47">
+      <c r="D3" s="56">
         <v>0.99450000000000005</v>
       </c>
-      <c r="E3" s="47" t="s">
+      <c r="E3" s="56" t="s">
         <v>75</v>
       </c>
-      <c r="F3" s="47" t="s">
+      <c r="F3" s="56" t="s">
         <v>97</v>
       </c>
-      <c r="G3" s="47">
+      <c r="G3" s="56">
         <v>0.98540000000000005</v>
       </c>
-      <c r="H3" s="47" t="s">
+      <c r="H3" s="56" t="s">
         <v>89</v>
       </c>
-      <c r="I3" s="47" t="s">
+      <c r="I3" s="56" t="s">
         <v>70</v>
       </c>
       <c r="J3" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="4" spans="1:10" ht="28.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="48"/>
+    <row r="4" spans="1:10" ht="28.15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="57"/>
       <c r="B4" s="15" t="s">
         <v>68</v>
       </c>
       <c r="C4" s="16" t="s">
         <v>72</v>
       </c>
-      <c r="D4" s="48"/>
-      <c r="E4" s="48"/>
-      <c r="F4" s="48"/>
-      <c r="G4" s="48"/>
-      <c r="H4" s="48"/>
-      <c r="I4" s="48"/>
-    </row>
-    <row r="5" spans="1:10" ht="28.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="25" t="s">
+      <c r="D4" s="57"/>
+      <c r="E4" s="57"/>
+      <c r="F4" s="57"/>
+      <c r="G4" s="57"/>
+      <c r="H4" s="57"/>
+      <c r="I4" s="57"/>
+    </row>
+    <row r="5" spans="1:10" ht="28.15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="40" t="s">
         <v>6</v>
       </c>
       <c r="B5" s="9" t="s">
@@ -2267,45 +2266,45 @@
       <c r="C5" s="11" t="s">
         <v>73</v>
       </c>
-      <c r="D5" s="27">
+      <c r="D5" s="36">
         <v>0.98540000000000005</v>
       </c>
-      <c r="E5" s="27" t="s">
+      <c r="E5" s="36" t="s">
         <v>69</v>
       </c>
-      <c r="F5" s="27" t="s">
+      <c r="F5" s="36" t="s">
         <v>70</v>
       </c>
-      <c r="G5" s="27" t="s">
+      <c r="G5" s="36" t="s">
         <v>4</v>
       </c>
-      <c r="H5" s="49" t="s">
+      <c r="H5" s="58" t="s">
         <v>91</v>
       </c>
-      <c r="I5" s="49" t="s">
+      <c r="I5" s="58" t="s">
         <v>92</v>
       </c>
       <c r="J5" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="6" spans="1:10" ht="28.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="26"/>
+    <row r="6" spans="1:10" ht="28.15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="42"/>
       <c r="B6" s="10" t="s">
         <v>94</v>
       </c>
       <c r="C6" s="12" t="s">
         <v>74</v>
       </c>
-      <c r="D6" s="28"/>
-      <c r="E6" s="28"/>
-      <c r="F6" s="28"/>
-      <c r="G6" s="26"/>
-      <c r="H6" s="50"/>
-      <c r="I6" s="50"/>
-    </row>
-    <row r="7" spans="1:10" ht="28.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="25" t="s">
+      <c r="D6" s="38"/>
+      <c r="E6" s="38"/>
+      <c r="F6" s="38"/>
+      <c r="G6" s="42"/>
+      <c r="H6" s="59"/>
+      <c r="I6" s="59"/>
+    </row>
+    <row r="7" spans="1:10" ht="28.15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="40" t="s">
         <v>10</v>
       </c>
       <c r="B7" s="9" t="s">
@@ -2314,44 +2313,44 @@
       <c r="C7" s="11" t="s">
         <v>85</v>
       </c>
-      <c r="D7" s="25">
+      <c r="D7" s="40">
         <v>0.99450000000000005</v>
       </c>
-      <c r="E7" s="25" t="s">
+      <c r="E7" s="40" t="s">
         <v>103</v>
       </c>
-      <c r="F7" s="25" t="s">
+      <c r="F7" s="40" t="s">
         <v>86</v>
       </c>
-      <c r="G7" s="27" t="s">
+      <c r="G7" s="36" t="s">
         <v>4</v>
       </c>
-      <c r="H7" s="27" t="s">
+      <c r="H7" s="36" t="s">
         <v>90</v>
       </c>
-      <c r="I7" s="27" t="s">
+      <c r="I7" s="36" t="s">
         <v>88</v>
       </c>
       <c r="J7" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="8" spans="1:10" ht="28.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="26"/>
+    <row r="8" spans="1:10" ht="28.15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="42"/>
       <c r="B8" s="10" t="s">
         <v>96</v>
       </c>
       <c r="C8" s="12" t="s">
         <v>84</v>
       </c>
-      <c r="D8" s="26"/>
-      <c r="E8" s="26"/>
-      <c r="F8" s="26"/>
-      <c r="G8" s="26"/>
-      <c r="H8" s="26"/>
-      <c r="I8" s="26"/>
-    </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="D8" s="42"/>
+      <c r="E8" s="42"/>
+      <c r="F8" s="42"/>
+      <c r="G8" s="42"/>
+      <c r="H8" s="42"/>
+      <c r="I8" s="42"/>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>98</v>
       </c>
@@ -2359,7 +2358,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>99</v>
       </c>
@@ -2378,16 +2377,6 @@
     </row>
   </sheetData>
   <mergeCells count="26">
-    <mergeCell ref="A3:A4"/>
-    <mergeCell ref="A5:A6"/>
-    <mergeCell ref="D5:D6"/>
-    <mergeCell ref="E5:E6"/>
-    <mergeCell ref="F5:F6"/>
-    <mergeCell ref="A1:A2"/>
-    <mergeCell ref="D1:F1"/>
-    <mergeCell ref="B1:B2"/>
-    <mergeCell ref="C1:C2"/>
-    <mergeCell ref="G1:I1"/>
     <mergeCell ref="G3:G4"/>
     <mergeCell ref="H3:H4"/>
     <mergeCell ref="I7:I8"/>
@@ -2404,6 +2393,16 @@
     <mergeCell ref="D3:D4"/>
     <mergeCell ref="E3:E4"/>
     <mergeCell ref="F3:F4"/>
+    <mergeCell ref="A1:A2"/>
+    <mergeCell ref="D1:F1"/>
+    <mergeCell ref="B1:B2"/>
+    <mergeCell ref="C1:C2"/>
+    <mergeCell ref="G1:I1"/>
+    <mergeCell ref="A3:A4"/>
+    <mergeCell ref="A5:A6"/>
+    <mergeCell ref="D5:D6"/>
+    <mergeCell ref="E5:E6"/>
+    <mergeCell ref="F5:F6"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -2412,40 +2411,40 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{959911B6-8118-467B-8966-D274265204EE}">
   <dimension ref="A1:J10"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="8.88671875" style="3"/>
-    <col min="2" max="2" width="10.6640625" style="3" customWidth="1"/>
-    <col min="3" max="3" width="5.6640625" customWidth="1"/>
+    <col min="1" max="1" width="8.85546875" style="3"/>
+    <col min="2" max="2" width="10.7109375" style="3" customWidth="1"/>
+    <col min="3" max="3" width="5.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="52" t="s">
+    <row r="1" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="63" t="s">
         <v>141</v>
       </c>
-      <c r="B1" s="52"/>
-      <c r="C1" s="52" t="s">
+      <c r="B1" s="63"/>
+      <c r="C1" s="63" t="s">
         <v>142</v>
       </c>
-      <c r="D1" s="52" t="s">
+      <c r="D1" s="63" t="s">
         <v>143</v>
       </c>
-      <c r="E1" s="51" t="s">
+      <c r="E1" s="60" t="s">
         <v>147</v>
       </c>
-      <c r="F1" s="51"/>
-      <c r="G1" s="51"/>
-      <c r="H1" s="51" t="s">
+      <c r="F1" s="60"/>
+      <c r="G1" s="60"/>
+      <c r="H1" s="60" t="s">
         <v>148</v>
       </c>
-      <c r="I1" s="51"/>
-      <c r="J1" s="51"/>
-    </row>
-    <row r="2" spans="1:10" s="3" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="52"/>
-      <c r="B2" s="52"/>
-      <c r="C2" s="52"/>
-      <c r="D2" s="52"/>
+      <c r="I1" s="60"/>
+      <c r="J1" s="60"/>
+    </row>
+    <row r="2" spans="1:10" s="3" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="63"/>
+      <c r="B2" s="63"/>
+      <c r="C2" s="63"/>
+      <c r="D2" s="63"/>
       <c r="E2" s="20" t="s">
         <v>146</v>
       </c>
@@ -2465,11 +2464,11 @@
         <v>145</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A3" s="53" t="s">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A3" s="61" t="s">
         <v>138</v>
       </c>
-      <c r="B3" s="54" t="s">
+      <c r="B3" s="62" t="s">
         <v>139</v>
       </c>
       <c r="C3" s="18">
@@ -2497,9 +2496,9 @@
         <v>3.2421000000000002</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A4" s="53"/>
-      <c r="B4" s="54"/>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A4" s="61"/>
+      <c r="B4" s="62"/>
       <c r="C4" s="18">
         <v>10</v>
       </c>
@@ -2525,9 +2524,9 @@
         <v>4.6946000000000003</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A5" s="53"/>
-      <c r="B5" s="54" t="s">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A5" s="61"/>
+      <c r="B5" s="62" t="s">
         <v>140</v>
       </c>
       <c r="C5" s="18">
@@ -2555,9 +2554,9 @@
         <v>1.0546</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A6" s="53"/>
-      <c r="B6" s="54"/>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A6" s="61"/>
+      <c r="B6" s="62"/>
       <c r="C6" s="18">
         <v>20</v>
       </c>
@@ -2583,11 +2582,11 @@
         <v>3.5497999999999998</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A7" s="53" t="s">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A7" s="61" t="s">
         <v>149</v>
       </c>
-      <c r="B7" s="51" t="s">
+      <c r="B7" s="60" t="s">
         <v>139</v>
       </c>
       <c r="C7" s="18">
@@ -2615,9 +2614,9 @@
         <v>3.58761452437188</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A8" s="53"/>
-      <c r="B8" s="51"/>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A8" s="61"/>
+      <c r="B8" s="60"/>
       <c r="C8" s="18">
         <v>10</v>
       </c>
@@ -2643,9 +2642,9 @@
         <v>1.8463910818920899</v>
       </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A9" s="53"/>
-      <c r="B9" s="51"/>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A9" s="61"/>
+      <c r="B9" s="60"/>
       <c r="C9" s="18">
         <v>10</v>
       </c>
@@ -2671,8 +2670,8 @@
         <v>2.0676835787835999</v>
       </c>
     </row>
-    <row r="10" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A10" s="53"/>
+    <row r="10" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A10" s="61"/>
       <c r="B10" s="19" t="s">
         <v>140</v>
       </c>
@@ -2703,16 +2702,16 @@
     </row>
   </sheetData>
   <mergeCells count="10">
+    <mergeCell ref="E1:G1"/>
+    <mergeCell ref="H1:J1"/>
+    <mergeCell ref="A1:B2"/>
+    <mergeCell ref="C1:C2"/>
+    <mergeCell ref="D1:D2"/>
     <mergeCell ref="B7:B9"/>
     <mergeCell ref="A7:A10"/>
     <mergeCell ref="A3:A6"/>
     <mergeCell ref="B3:B4"/>
     <mergeCell ref="B5:B6"/>
-    <mergeCell ref="E1:G1"/>
-    <mergeCell ref="H1:J1"/>
-    <mergeCell ref="A1:B2"/>
-    <mergeCell ref="C1:C2"/>
-    <mergeCell ref="D1:D2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -2721,12 +2720,12 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{07F20C50-7E80-41CF-971C-9DF8CC7EC325}">
   <dimension ref="A1:E3"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="9.109375" style="3"/>
+    <col min="1" max="1" width="9.140625" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="21"/>
       <c r="B1" s="21" t="s">
         <v>150</v>
@@ -2741,7 +2740,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="21" t="s">
         <v>138</v>
       </c>
@@ -2758,7 +2757,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="21" t="s">
         <v>149</v>
       </c>
@@ -2784,261 +2783,261 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{89E6C615-F30D-46B6-996B-A5B4C010E31A}">
   <dimension ref="A1:K8"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A1" s="55" t="s">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1" s="25" t="s">
         <v>155</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>156</v>
       </c>
-      <c r="C1" s="55"/>
-      <c r="D1" s="56" t="s">
+      <c r="C1" s="25"/>
+      <c r="D1" s="26" t="s">
         <v>157</v>
       </c>
-      <c r="E1" s="57"/>
-      <c r="F1" s="55"/>
-      <c r="G1" s="56" t="s">
+      <c r="E1" s="27"/>
+      <c r="F1" s="25"/>
+      <c r="G1" s="26" t="s">
         <v>158</v>
       </c>
-      <c r="H1" s="57"/>
-      <c r="I1" s="55"/>
-      <c r="J1" s="56" t="s">
+      <c r="H1" s="27"/>
+      <c r="I1" s="25"/>
+      <c r="J1" s="26" t="s">
         <v>165</v>
       </c>
-      <c r="K1" s="57"/>
-    </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A2" s="58"/>
-      <c r="B2" s="64"/>
-      <c r="C2" s="61" t="s">
+      <c r="K1" s="27"/>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A2" s="28"/>
+      <c r="B2" s="33"/>
+      <c r="C2" s="30" t="s">
         <v>2</v>
       </c>
-      <c r="D2" s="62" t="s">
+      <c r="D2" s="31" t="s">
         <v>144</v>
       </c>
-      <c r="E2" s="63" t="s">
+      <c r="E2" s="32" t="s">
         <v>14</v>
       </c>
-      <c r="F2" s="61" t="s">
+      <c r="F2" s="30" t="s">
         <v>2</v>
       </c>
-      <c r="G2" s="62" t="s">
+      <c r="G2" s="31" t="s">
         <v>144</v>
       </c>
-      <c r="H2" s="63" t="s">
+      <c r="H2" s="32" t="s">
         <v>164</v>
       </c>
-      <c r="I2" s="61" t="s">
+      <c r="I2" s="30" t="s">
         <v>2</v>
       </c>
-      <c r="J2" s="62" t="s">
+      <c r="J2" s="31" t="s">
         <v>144</v>
       </c>
-      <c r="K2" s="63" t="s">
+      <c r="K2" s="32" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A3" s="55" t="s">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A3" s="25" t="s">
         <v>159</v>
       </c>
       <c r="B3" s="1" t="s">
         <v>161</v>
       </c>
-      <c r="C3" s="58">
+      <c r="C3" s="28">
         <v>10.030023297662</v>
       </c>
-      <c r="D3" s="59">
+      <c r="D3">
         <v>5.7857520576062599E-3</v>
       </c>
-      <c r="E3" s="60">
+      <c r="E3" s="29">
         <v>39.1683403041486</v>
       </c>
-      <c r="F3" s="58">
+      <c r="F3" s="28">
         <v>140.919546217841</v>
       </c>
-      <c r="G3" s="59">
+      <c r="G3">
         <v>1.1420849455901001</v>
       </c>
-      <c r="H3" s="60">
+      <c r="H3" s="29">
         <v>278.293987665835</v>
       </c>
-      <c r="I3" s="58">
+      <c r="I3" s="28">
         <v>230.92279507222699</v>
       </c>
-      <c r="J3" s="59">
+      <c r="J3">
         <v>3.0668288914488202</v>
       </c>
-      <c r="K3" s="60">
+      <c r="K3" s="29">
         <v>366.67664917371502</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A4" s="58"/>
-      <c r="B4" s="64" t="s">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A4" s="28"/>
+      <c r="B4" s="33" t="s">
         <v>162</v>
       </c>
-      <c r="C4" s="58">
+      <c r="C4" s="28">
         <v>11.4768172384107</v>
       </c>
-      <c r="D4" s="59">
+      <c r="D4">
         <v>5.7857520576062599E-3</v>
       </c>
-      <c r="E4" s="60">
+      <c r="E4" s="29">
         <v>44.818229216613403</v>
       </c>
-      <c r="F4" s="58">
+      <c r="F4" s="28">
         <v>111.656768550769</v>
       </c>
-      <c r="G4" s="59">
+      <c r="G4">
         <v>0.54762970374824205</v>
       </c>
-      <c r="H4" s="60">
+      <c r="H4" s="29">
         <v>230.12450415175101</v>
       </c>
-      <c r="I4" s="58">
+      <c r="I4" s="28">
         <v>55.255628085825499</v>
       </c>
-      <c r="J4" s="59">
+      <c r="J4">
         <v>0.13411270636696501</v>
       </c>
-      <c r="K4" s="60">
+      <c r="K4" s="29">
         <v>117.90686694998701</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A5" s="58"/>
-      <c r="B5" s="64" t="s">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A5" s="28"/>
+      <c r="B5" s="33" t="s">
         <v>163</v>
       </c>
-      <c r="C5" s="58">
+      <c r="C5" s="28">
         <v>11.967721487108101</v>
       </c>
-      <c r="D5" s="59">
+      <c r="D5">
         <v>5.7857520576062599E-3</v>
       </c>
-      <c r="E5" s="60">
+      <c r="E5" s="29">
         <v>46.735264112655301</v>
       </c>
-      <c r="F5" s="58">
+      <c r="F5" s="28">
         <v>101.780464999041</v>
       </c>
-      <c r="G5" s="59">
+      <c r="G5">
         <v>0.41847135223887799</v>
       </c>
-      <c r="H5" s="60">
+      <c r="H5" s="29">
         <v>213.780363186946</v>
       </c>
-      <c r="I5" s="58">
+      <c r="I5" s="28">
         <v>792.79480354758095</v>
       </c>
-      <c r="J5" s="59">
+      <c r="J5">
         <v>25.389752110895</v>
       </c>
-      <c r="K5" s="60">
+      <c r="K5" s="29">
         <v>1233.3510949634499</v>
       </c>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A6" s="55" t="s">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A6" s="25" t="s">
         <v>160</v>
       </c>
       <c r="B6" s="1" t="s">
         <v>161</v>
       </c>
-      <c r="C6" s="55">
+      <c r="C6" s="25">
         <v>24.047151878093999</v>
       </c>
-      <c r="D6" s="56">
+      <c r="D6" s="26">
         <v>7.2794745392710698E-3</v>
       </c>
-      <c r="E6" s="57">
+      <c r="E6" s="27">
         <v>71.271359058105901</v>
       </c>
-      <c r="F6" s="55">
+      <c r="F6" s="25">
         <v>270.82008047220802</v>
       </c>
-      <c r="G6" s="56">
+      <c r="G6" s="26">
         <v>0.92328220312534903</v>
       </c>
-      <c r="H6" s="57">
+      <c r="H6" s="27">
         <v>658.87715147126903</v>
       </c>
-      <c r="I6" s="55">
+      <c r="I6" s="25">
         <v>896.06222516664604</v>
       </c>
-      <c r="J6" s="56">
+      <c r="J6" s="26">
         <v>10.1076239892818</v>
       </c>
-      <c r="K6" s="57">
+      <c r="K6" s="27">
         <v>1345.61019986718</v>
       </c>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A7" s="58"/>
-      <c r="B7" s="64" t="s">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A7" s="28"/>
+      <c r="B7" s="33" t="s">
         <v>162</v>
       </c>
-      <c r="C7" s="58">
+      <c r="C7" s="28">
         <v>28.453462927716998</v>
       </c>
-      <c r="D7" s="59">
+      <c r="D7">
         <v>7.2794745392710698E-3</v>
       </c>
-      <c r="E7" s="60">
+      <c r="E7" s="29">
         <v>84.330858932827496</v>
       </c>
-      <c r="F7" s="58">
+      <c r="F7" s="28">
         <v>225.70164180492799</v>
       </c>
-      <c r="G7" s="59">
+      <c r="G7">
         <v>0.45803557290533597</v>
       </c>
-      <c r="H7" s="60">
+      <c r="H7" s="29">
         <v>525.49531413858301</v>
       </c>
-      <c r="I7" s="58">
+      <c r="I7" s="28">
         <v>54.912251149549597</v>
       </c>
-      <c r="J7" s="59">
+      <c r="J7">
         <v>2.7112419040766299E-2</v>
       </c>
-      <c r="K7" s="60">
+      <c r="K7" s="29">
         <v>131.68077924574499</v>
       </c>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A8" s="61"/>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A8" s="30"/>
       <c r="B8" s="2" t="s">
         <v>163</v>
       </c>
-      <c r="C8" s="61">
+      <c r="C8" s="30">
         <v>29.986771161392699</v>
       </c>
-      <c r="D8" s="62">
+      <c r="D8" s="31">
         <v>7.2794745392710698E-3</v>
       </c>
-      <c r="E8" s="63">
+      <c r="E8" s="32">
         <v>88.875304038969205</v>
       </c>
-      <c r="F8" s="61">
+      <c r="F8" s="30">
         <v>200.831158864316</v>
       </c>
-      <c r="G8" s="62">
+      <c r="G8" s="31">
         <v>0.32651475316463502</v>
       </c>
-      <c r="H8" s="63">
+      <c r="H8" s="32">
         <v>460.86727263098902</v>
       </c>
-      <c r="I8" s="61">
+      <c r="I8" s="30">
         <v>827.56952601990804</v>
       </c>
-      <c r="J8" s="62">
+      <c r="J8" s="31">
         <v>5.5443367526663696</v>
       </c>
-      <c r="K8" s="63">
+      <c r="K8" s="32">
         <v>1329.8883440250199</v>
       </c>
     </row>

</xml_diff>